<commit_message>
Fix translation logic and update cleaned_quotes.xlsx
</commit_message>
<xml_diff>
--- a/cleaned_quotes.xlsx
+++ b/cleaned_quotes.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D11"/>
+  <dimension ref="A1:E11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -424,15 +424,20 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>Quote Text</t>
+          <t>Quote Text (Eng)</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
+          <t>Quote Text (MM)</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
           <t>Author</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Tags</t>
         </is>
@@ -444,15 +449,20 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>The world as we have created it is a process of our thinking. It cannot be changed without changing our thinking.</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
+          <t>ငါတို့ဖန်တီးထားတဲ့ ကမ္ဘာကြီးဟာ ငါတို့ရဲ့ တွေးခေါ်မှုဖြစ်စဉ်တစ်ခုပါ။ ကျွန်တော်တို့ရဲ့ တွေးခေါ်ပုံကို မပြောင်းလဲဘဲ ပြောင်းလဲလို့ မရပါဘူး။</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
           <t>Albert Einstein</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="E2" t="inlineStr">
         <is>
           <t>change, deep-thoughts, thinking, world</t>
         </is>
@@ -464,15 +474,20 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>It is our choices, Harry, that show what we truly are, far more than our abilities.</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
+          <t>ဟယ်ရီ၊ ငါတို့ရဲ့ အရည်အချင်းတွေထက် ငါတို့အမှန်တကယ်ရှိတာကို ပြသတဲ့ ငါတို့ရဲ့ ရွေးချယ်မှုပဲ။</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
           <t>J.K. Rowling</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="E3" t="inlineStr">
         <is>
           <t>abilities, choices</t>
         </is>
@@ -484,15 +499,20 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>There are only two ways to live your life. One is as though nothing is a miracle. The other is as though everything is a miracle.</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
+          <t>သင့်ဘဝနေထိုင်ရန် နည်းလမ်းနှစ်ခုသာရှိသည်။ တစ်ခုက ဘာမှ အံ့ဖွယ်မရှိသလိုပဲ။ နောက်တစ်ခုက အရာအားလုံးဟာ အံ့ဖွယ်တစ်ခုလိုပါပဲ။</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
           <t>Albert Einstein</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="E4" t="inlineStr">
         <is>
           <t>inspirational, life, live, miracle, miracles</t>
         </is>
@@ -504,15 +524,20 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>The person, be it gentleman or lady, who has not pleasure in a good novel, must be intolerably stupid.</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
+          <t>ကောင်းသောဝတ္ထု၌ မနှစ်သက်သော အမျိုးကောင်းသားဖြစ်စေ၊ မိန်းမဖြစ်စေ ၊</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
           <t>Jane Austen</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="E5" t="inlineStr">
         <is>
           <t>aliteracy, books, classic, humor</t>
         </is>
@@ -524,15 +549,20 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Imperfection is beauty, madness is genius and it's better to be absolutely ridiculous than absolutely boring.</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
+          <t>မစုံလင်မှုသည် အလှတရား၊ ရူးသွပ်ခြင်းသည် ဉာဏ်ကြီးရှင်ဖြစ်ပြီး ပျင်းစရာကောင်းသည်ထက် လုံးဝရယ်စရာကောင်းသည်။</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
           <t>Marilyn Monroe</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
+      <c r="E6" t="inlineStr">
         <is>
           <t>be-yourself, inspirational</t>
         </is>
@@ -544,15 +574,20 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Try not to become a man of success. Rather become a man of value.</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
+          <t>အောင်မြင်သူတစ်ယောက်ဖြစ်ဖို့ မကြိုးစားပါနဲ့။ တန်ဖိုးထားတတ်သူဖြစ်ပါစေ။</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
           <t>Albert Einstein</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
+      <c r="E7" t="inlineStr">
         <is>
           <t>adulthood, success, value</t>
         </is>
@@ -564,15 +599,20 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>It is better to be hated for what you are than to be loved for what you are not.</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
+          <t>ကိုယ်မဟုတ်တဲ့အရာအတွက် ချစ်တာထက် မုန်းတီးတာက ပိုကောင်းပါတယ်။</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
           <t>André Gide</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
+      <c r="E8" t="inlineStr">
         <is>
           <t>life, love</t>
         </is>
@@ -584,15 +624,20 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>I have not failed. I've just found 10,000 ways that won't work.</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
+          <t>ငါမအောင်မြင်ဘူး။ အလုပ်မဖြစ်နိုင်တဲ့ နည်းလမ်း 10,000 လောက်ကို ရှာတွေ့ခဲ့ပါတယ်။</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
           <t>Thomas A. Edison</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr">
+      <c r="E9" t="inlineStr">
         <is>
           <t>edison, failure, inspirational, paraphrased</t>
         </is>
@@ -604,15 +649,20 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>A woman is like a tea bag; you never know how strong it is until it's in hot water.</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
+          <t>Error 500 (Server Error)!!1500.That’s an error.There was an error. Please try again later.That’s all we know.</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
           <t>Eleanor Roosevelt</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr">
+      <c r="E10" t="inlineStr">
         <is>
           <t>misattributed-eleanor-roosevelt</t>
         </is>
@@ -624,15 +674,20 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>A day without sunshine is like, you know, night.</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
+          <t>နေရောင်ခြည်မရှိသောနေ့သည် ညနှင့်တူသည်။</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
           <t>Steve Martin</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr">
+      <c r="E11" t="inlineStr">
         <is>
           <t>humor, obvious, simile</t>
         </is>

</xml_diff>

<commit_message>
Complete Lesson 20: Multi-page web scraping with error handling
</commit_message>
<xml_diff>
--- a/cleaned_quotes.xlsx
+++ b/cleaned_quotes.xlsx
@@ -454,7 +454,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>ငါတို့ဖန်တီးထားတဲ့ ကမ္ဘာကြီးဟာ ငါတို့ရဲ့ တွေးခေါ်မှုဖြစ်စဉ်တစ်ခုပါ။ ကျွန်တော်တို့ရဲ့ တွေးခေါ်ပုံကို မပြောင်းလဲဘဲ ပြောင်းလဲလို့ မရပါဘူး။</t>
+          <t>Error 500 (Server Error)!!1500.That’s an error.There was an error. Please try again later.That’s all we know.</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -479,7 +479,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>ဟယ်ရီ၊ ငါတို့ရဲ့ အရည်အချင်းတွေထက် ငါတို့အမှန်တကယ်ရှိတာကို ပြသတဲ့ ငါတို့ရဲ့ ရွေးချယ်မှုပဲ။</t>
+          <t>Error 500 (Server Error)!!1500.That’s an error.There was an error. Please try again later.That’s all we know.</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -504,7 +504,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>သင့်ဘဝနေထိုင်ရန် နည်းလမ်းနှစ်ခုသာရှိသည်။ တစ်ခုက ဘာမှ အံ့ဖွယ်မရှိသလိုပဲ။ နောက်တစ်ခုက အရာအားလုံးဟာ အံ့ဖွယ်တစ်ခုလိုပါပဲ။</t>
+          <t>Error 500 (Server Error)!!1500.That’s an error.There was an error. Please try again later.That’s all we know.</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -529,7 +529,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>ကောင်းသောဝတ္ထု၌ မနှစ်သက်သော အမျိုးကောင်းသားဖြစ်စေ၊ မိန်းမဖြစ်စေ ၊</t>
+          <t>Error 500 (Server Error)!!1500.That’s an error.There was an error. Please try again later.That’s all we know.</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -554,7 +554,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>မစုံလင်မှုသည် အလှတရား၊ ရူးသွပ်ခြင်းသည် ဉာဏ်ကြီးရှင်ဖြစ်ပြီး ပျင်းစရာကောင်းသည်ထက် လုံးဝရယ်စရာကောင်းသည်။</t>
+          <t>Error 500 (Server Error)!!1500.That’s an error.There was an error. Please try again later.That’s all we know.</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -579,7 +579,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>အောင်မြင်သူတစ်ယောက်ဖြစ်ဖို့ မကြိုးစားပါနဲ့။ တန်ဖိုးထားတတ်သူဖြစ်ပါစေ။</t>
+          <t>Error 500 (Server Error)!!1500.That’s an error.There was an error. Please try again later.That’s all we know.</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -604,7 +604,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>ကိုယ်မဟုတ်တဲ့အရာအတွက် ချစ်တာထက် မုန်းတီးတာက ပိုကောင်းပါတယ်။</t>
+          <t>Error 500 (Server Error)!!1500.That’s an error.There was an error. Please try again later.That’s all we know.</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -629,7 +629,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>ငါမအောင်မြင်ဘူး။ အလုပ်မဖြစ်နိုင်တဲ့ နည်းလမ်း 10,000 လောက်ကို ရှာတွေ့ခဲ့ပါတယ်။</t>
+          <t>Error 500 (Server Error)!!1500.That’s an error.There was an error. Please try again later.That’s all we know.</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -679,7 +679,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>နေရောင်ခြည်မရှိသောနေ့သည် ညနှင့်တူသည်။</t>
+          <t>Error 500 (Server Error)!!1500.That’s an error.There was an error. Please try again later.That’s all we know.</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">

</xml_diff>